<commit_message>
feat(readme) :Ajoute de l'affichage du contenu des livres
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_DamienChabal.xlsx
+++ b/Journal-de-Travail_DamienChabal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\P_AppMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5341B8D-2D1F-456B-9183-41641AA2451C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45D63359-BD8F-47D2-9B33-B00C42B9F86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="33375" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t>Auteur:</t>
   </si>
@@ -143,6 +143,18 @@
   </si>
   <si>
     <t>Ajoute du du menu, la page de détail pour un livre</t>
+  </si>
+  <si>
+    <t>Ajoute de l'import d'un livre epub et affichage du livre dans la liste</t>
+  </si>
+  <si>
+    <t>Ajoute de la suppression d'un livre dans la liste</t>
+  </si>
+  <si>
+    <t>Amélioration des maquettes figma</t>
+  </si>
+  <si>
+    <t>Ajoute de l'affichage du contenu des livres</t>
   </si>
 </sst>
 </file>
@@ -1085,7 +1097,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>390</c:v>
+                  <c:v>575</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4178,7 +4190,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>6 heures 30 minutes</v>
+        <v>9 heures 35 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4191,15 +4203,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>390</v>
+        <v>575</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4345,15 +4357,25 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="74" t="str">
+      <c r="A11" s="74">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v/>
-      </c>
-      <c r="B11" s="40"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="28"/>
+        <v>17</v>
+      </c>
+      <c r="B11" s="40">
+        <v>46134</v>
+      </c>
+      <c r="C11" s="41">
+        <v>1</v>
+      </c>
+      <c r="D11" s="42">
+        <v>30</v>
+      </c>
+      <c r="E11" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>34</v>
+      </c>
       <c r="G11" s="46"/>
       <c r="M11" t="s">
         <v>4</v>
@@ -4366,15 +4388,23 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="73" t="str">
+      <c r="A12" s="73">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v/>
-      </c>
-      <c r="B12" s="36"/>
+        <v>17</v>
+      </c>
+      <c r="B12" s="36">
+        <v>46134</v>
+      </c>
       <c r="C12" s="37"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="28"/>
+      <c r="D12" s="38">
+        <v>25</v>
+      </c>
+      <c r="E12" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>35</v>
+      </c>
       <c r="G12" s="45"/>
       <c r="N12">
         <v>5</v>
@@ -4384,15 +4414,23 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="74" t="str">
+      <c r="A13" s="74">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="40"/>
+        <v>17</v>
+      </c>
+      <c r="B13" s="40">
+        <v>46134</v>
+      </c>
       <c r="C13" s="41"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="28"/>
+      <c r="D13" s="42">
+        <v>10</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>36</v>
+      </c>
       <c r="G13" s="46"/>
       <c r="N13">
         <v>6</v>
@@ -4402,15 +4440,23 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="73" t="str">
+      <c r="A14" s="73">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v/>
-      </c>
-      <c r="B14" s="36"/>
-      <c r="C14" s="37"/>
+        <v>18</v>
+      </c>
+      <c r="B14" s="36">
+        <v>46141</v>
+      </c>
+      <c r="C14" s="37">
+        <v>1</v>
+      </c>
       <c r="D14" s="38"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="28"/>
+      <c r="E14" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>37</v>
+      </c>
       <c r="G14" s="45"/>
       <c r="N14">
         <v>7</v>
@@ -10821,15 +10867,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>390</v>
+        <v>575</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10837,7 +10883,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>6 h 30 min</v>
+        <v>9 h 35 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -10932,26 +10978,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>390</v>
+        <v>575</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>6 h 30 min</v>
+        <v>9 h 35 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>7.3863636363636367E-2</v>
+        <v>0.10890151515151515</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
feat (readme) :Ajout de l'affichage des images du livres et debug de l'affichage avec du texte dans le livre
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_DamienChabal.xlsx
+++ b/Journal-de-Travail_DamienChabal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\P_AppMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45D63359-BD8F-47D2-9B33-B00C42B9F86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5185BE-3BC2-453A-A8FE-8BA1976EBF22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="33375" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
   <si>
     <t>Auteur:</t>
   </si>
@@ -142,19 +142,22 @@
     <t>Chabal Damien</t>
   </si>
   <si>
-    <t>Ajoute du du menu, la page de détail pour un livre</t>
-  </si>
-  <si>
-    <t>Ajoute de l'import d'un livre epub et affichage du livre dans la liste</t>
-  </si>
-  <si>
-    <t>Ajoute de la suppression d'un livre dans la liste</t>
-  </si>
-  <si>
     <t>Amélioration des maquettes figma</t>
   </si>
   <si>
-    <t>Ajoute de l'affichage du contenu des livres</t>
+    <t>Ajout de l'affichage du contenu des livres</t>
+  </si>
+  <si>
+    <t>Ajout de la suppression d'un livre dans la liste</t>
+  </si>
+  <si>
+    <t>Ajout de l'import d'un livre epub et affichage du livre dans la liste</t>
+  </si>
+  <si>
+    <t>Ajout du du menu, la page de détail pour un livre</t>
+  </si>
+  <si>
+    <t>Ajout de l'affichage des images du livres et debug de l'affichage avec du texte dans le livre</t>
   </si>
 </sst>
 </file>
@@ -1097,7 +1100,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>575</c:v>
+                  <c:v>665</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4190,7 +4193,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>9 heures 35 minutes</v>
+        <v>11 heures 5 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4203,15 +4206,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>575</v>
+        <v>665</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4343,7 +4346,7 @@
         <v>19</v>
       </c>
       <c r="F10" s="28" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G10" s="45"/>
       <c r="M10" t="s">
@@ -4374,7 +4377,7 @@
         <v>19</v>
       </c>
       <c r="F11" s="28" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G11" s="46"/>
       <c r="M11" t="s">
@@ -4429,7 +4432,7 @@
         <v>19</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G13" s="46"/>
       <c r="N13">
@@ -4450,12 +4453,14 @@
       <c r="C14" s="37">
         <v>1</v>
       </c>
-      <c r="D14" s="38"/>
+      <c r="D14" s="38">
+        <v>10</v>
+      </c>
       <c r="E14" s="39" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="28" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G14" s="45"/>
       <c r="N14">
@@ -4466,15 +4471,25 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="74" t="str">
+      <c r="A15" s="74">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="28"/>
+        <v>18</v>
+      </c>
+      <c r="B15" s="40">
+        <v>46141</v>
+      </c>
+      <c r="C15" s="41">
+        <v>1</v>
+      </c>
+      <c r="D15" s="42">
+        <v>20</v>
+      </c>
+      <c r="E15" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="28" t="s">
+        <v>38</v>
+      </c>
       <c r="G15" s="46"/>
       <c r="N15">
         <v>8</v>
@@ -10867,15 +10882,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>575</v>
+        <v>665</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10883,7 +10898,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>9 h 35 min</v>
+        <v>11 h 05 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -10978,26 +10993,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>575</v>
+        <v>665</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>9 h 35 min</v>
+        <v>11 h 05 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.10890151515151515</v>
+        <v>0.1259469696969697</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11036,18 +11051,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010080C9F2488912074FB587B9AD9ADAE5BB" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="020ab319e6f8d23aec07c29d6516d4ba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xmlns:ns3="eefa3612-053e-497a-ae76-8a76877f5e22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e15d3f914bf2a775f9387e5284d9197" ns2:_="" ns3:_="">
     <xsd:import namespace="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
@@ -11260,6 +11263,18 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11270,19 +11285,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6394C10-4386-493D-A99B-15992834CB10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11301,6 +11303,19 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
chore(readme) : maj du jdt
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_DamienChabal.xlsx
+++ b/Journal-de-Travail_DamienChabal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\P_AppMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5185BE-3BC2-453A-A8FE-8BA1976EBF22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDEC82AF-6EDE-476E-8E7E-89CD08FF0A3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33375" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="30750" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>Auteur:</t>
   </si>
@@ -158,6 +158,12 @@
   </si>
   <si>
     <t>Ajout de l'affichage des images du livres et debug de l'affichage avec du texte dans le livre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modification de la lecture pour que se soit page par page </t>
+  </si>
+  <si>
+    <t>Ajoute de la barre de progression dans un livre</t>
   </si>
 </sst>
 </file>
@@ -1100,7 +1106,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>665</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4193,7 +4199,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>11 heures 5 minutes</v>
+        <v>13 heures 5 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4206,7 +4212,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>480</v>
+        <v>600</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4214,7 +4220,7 @@
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>665</v>
+        <v>785</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4499,30 +4505,46 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="73" t="str">
+      <c r="A16" s="73">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="37"/>
+        <v>19</v>
+      </c>
+      <c r="B16" s="36">
+        <v>46148</v>
+      </c>
+      <c r="C16" s="37">
+        <v>1</v>
+      </c>
       <c r="D16" s="38"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="28"/>
+      <c r="E16" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>39</v>
+      </c>
       <c r="G16" s="45"/>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="74" t="str">
+      <c r="A17" s="74">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="41"/>
+        <v>19</v>
+      </c>
+      <c r="B17" s="40">
+        <v>46148</v>
+      </c>
+      <c r="C17" s="41">
+        <v>1</v>
+      </c>
       <c r="D17" s="42"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="28"/>
+      <c r="E17" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>40</v>
+      </c>
       <c r="G17" s="46"/>
       <c r="O17">
         <v>45</v>
@@ -10882,7 +10904,7 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>480</v>
+        <v>600</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
@@ -10890,7 +10912,7 @@
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>665</v>
+        <v>785</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10898,7 +10920,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>11 h 05 min</v>
+        <v>13 h 05 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -10993,7 +11015,7 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>480</v>
+        <v>600</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
@@ -11001,18 +11023,18 @@
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>665</v>
+        <v>785</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>11 h 05 min</v>
+        <v>13 h 05 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.1259469696969697</v>
+        <v>0.14867424242424243</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11051,6 +11073,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010080C9F2488912074FB587B9AD9ADAE5BB" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="020ab319e6f8d23aec07c29d6516d4ba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xmlns:ns3="eefa3612-053e-497a-ae76-8a76877f5e22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e15d3f914bf2a775f9387e5284d9197" ns2:_="" ns3:_="">
     <xsd:import namespace="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
@@ -11263,18 +11297,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11285,6 +11307,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6394C10-4386-493D-A99B-15992834CB10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11303,19 +11338,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat (readme) : ajout de la mémorisation de la page et reprise automatiquement a la bonne page
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_DamienChabal.xlsx
+++ b/Journal-de-Travail_DamienChabal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\P_AppMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDEC82AF-6EDE-476E-8E7E-89CD08FF0A3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E9198FD-5D1D-4727-9825-9DBB751FC8F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30750" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="6600" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="44">
   <si>
     <t>Auteur:</t>
   </si>
@@ -157,13 +157,22 @@
     <t>Ajout du du menu, la page de détail pour un livre</t>
   </si>
   <si>
-    <t>Ajout de l'affichage des images du livres et debug de l'affichage avec du texte dans le livre</t>
-  </si>
-  <si>
     <t xml:space="preserve">Modification de la lecture pour que se soit page par page </t>
   </si>
   <si>
-    <t>Ajoute de la barre de progression dans un livre</t>
+    <t>debug de l'affichage avec du texte dans le livre</t>
+  </si>
+  <si>
+    <t>Ajout de l'affichage des images du livres</t>
+  </si>
+  <si>
+    <t>Ajout de la barre de progression dans un livre</t>
+  </si>
+  <si>
+    <t>Ajout de la mémorisation de la page</t>
+  </si>
+  <si>
+    <t>Ajout de la reprise automatique a la bonne page dans un livre</t>
   </si>
 </sst>
 </file>
@@ -1106,7 +1115,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>785</c:v>
+                  <c:v>845</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4199,7 +4208,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>13 heures 5 minutes</v>
+        <v>14 heures 5 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4216,11 +4225,11 @@
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>185</v>
+        <v>245</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>785</v>
+        <v>845</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4487,14 +4496,12 @@
       <c r="C15" s="41">
         <v>1</v>
       </c>
-      <c r="D15" s="42">
-        <v>20</v>
-      </c>
+      <c r="D15" s="42"/>
       <c r="E15" s="43" t="s">
         <v>19</v>
       </c>
       <c r="F15" s="28" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G15" s="46"/>
       <c r="N15">
@@ -4507,15 +4514,15 @@
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="73">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" s="36">
-        <v>46148</v>
-      </c>
-      <c r="C16" s="37">
-        <v>1</v>
-      </c>
-      <c r="D16" s="38"/>
+        <v>46141</v>
+      </c>
+      <c r="C16" s="37"/>
+      <c r="D16" s="38">
+        <v>20</v>
+      </c>
       <c r="E16" s="39" t="s">
         <v>19</v>
       </c>
@@ -4543,7 +4550,7 @@
         <v>19</v>
       </c>
       <c r="F17" s="28" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G17" s="46"/>
       <c r="O17">
@@ -4551,45 +4558,69 @@
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="73" t="str">
+      <c r="A18" s="73">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="37"/>
+        <v>19</v>
+      </c>
+      <c r="B18" s="36">
+        <v>46148</v>
+      </c>
+      <c r="C18" s="37">
+        <v>1</v>
+      </c>
       <c r="D18" s="38"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="28"/>
+      <c r="E18" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>41</v>
+      </c>
       <c r="G18" s="45"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="74" t="str">
+      <c r="A19" s="74">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="40"/>
+        <v>20</v>
+      </c>
+      <c r="B19" s="40">
+        <v>46155</v>
+      </c>
       <c r="C19" s="41"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="28"/>
+      <c r="D19" s="42">
+        <v>45</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="28" t="s">
+        <v>42</v>
+      </c>
       <c r="G19" s="46"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="73" t="str">
+      <c r="A20" s="73">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="36"/>
+        <v>20</v>
+      </c>
+      <c r="B20" s="36">
+        <v>46155</v>
+      </c>
       <c r="C20" s="37"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="28"/>
+      <c r="D20" s="38">
+        <v>15</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>43</v>
+      </c>
       <c r="G20" s="45"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -10908,11 +10939,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>185</v>
+        <v>245</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>785</v>
+        <v>845</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10920,7 +10951,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>13 h 05 min</v>
+        <v>14 h 05 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -11019,22 +11050,22 @@
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>185</v>
+        <v>245</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>785</v>
+        <v>845</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>13 h 05 min</v>
+        <v>14 h 05 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.14867424242424243</v>
+        <v>0.16003787878787878</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
feat(readme) : Ajout du tri par date
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_DamienChabal.xlsx
+++ b/Journal-de-Travail_DamienChabal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\P_AppMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E9198FD-5D1D-4727-9825-9DBB751FC8F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22BFAB30-948C-4456-BCAB-C75DE56BA61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6600" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
   <si>
     <t>Auteur:</t>
   </si>
@@ -173,6 +173,9 @@
   </si>
   <si>
     <t>Ajout de la reprise automatique a la bonne page dans un livre</t>
+  </si>
+  <si>
+    <t>Ajout du tri par date</t>
   </si>
 </sst>
 </file>
@@ -1115,7 +1118,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>845</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4208,7 +4211,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>14 heures 5 minutes</v>
+        <v>15 heures 0 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4221,15 +4224,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>600</v>
+        <v>660</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>845</v>
+        <v>900</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4588,10 +4591,10 @@
       <c r="B19" s="40">
         <v>46155</v>
       </c>
-      <c r="C19" s="41"/>
-      <c r="D19" s="42">
-        <v>45</v>
-      </c>
+      <c r="C19" s="41">
+        <v>1</v>
+      </c>
+      <c r="D19" s="42"/>
       <c r="E19" s="43" t="s">
         <v>19</v>
       </c>
@@ -4613,7 +4616,7 @@
       </c>
       <c r="C20" s="37"/>
       <c r="D20" s="38">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E20" s="39" t="s">
         <v>19</v>
@@ -4624,15 +4627,23 @@
       <c r="G20" s="45"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="74" t="str">
+      <c r="A21" s="74">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="40"/>
+        <v>20</v>
+      </c>
+      <c r="B21" s="40">
+        <v>46155</v>
+      </c>
       <c r="C21" s="41"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="28"/>
+      <c r="D21" s="42">
+        <v>30</v>
+      </c>
+      <c r="E21" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" s="28" t="s">
+        <v>44</v>
+      </c>
       <c r="G21" s="46"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -10935,15 +10946,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>600</v>
+        <v>660</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>845</v>
+        <v>900</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10951,7 +10962,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>14 h 05 min</v>
+        <v>15 h 00 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -11046,26 +11057,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>600</v>
+        <v>660</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>845</v>
+        <v>900</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>14 h 05 min</v>
+        <v>15 h 00 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.16003787878787878</v>
+        <v>0.17045454545454544</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11104,18 +11115,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010080C9F2488912074FB587B9AD9ADAE5BB" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="020ab319e6f8d23aec07c29d6516d4ba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xmlns:ns3="eefa3612-053e-497a-ae76-8a76877f5e22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e15d3f914bf2a775f9387e5284d9197" ns2:_="" ns3:_="">
     <xsd:import namespace="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
@@ -11328,6 +11327,18 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11338,19 +11349,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6394C10-4386-493D-A99B-15992834CB10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11369,6 +11367,19 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
chore (readme) : maj du jdt
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_DamienChabal.xlsx
+++ b/Journal-de-Travail_DamienChabal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\P_AppMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22BFAB30-948C-4456-BCAB-C75DE56BA61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B5BBE0-5299-409B-931F-F01208E9B5B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6600" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="46">
   <si>
     <t>Auteur:</t>
   </si>
@@ -176,6 +176,9 @@
   </si>
   <si>
     <t>Ajout du tri par date</t>
+  </si>
+  <si>
+    <t>meilleur affichage</t>
   </si>
 </sst>
 </file>
@@ -1118,7 +1121,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>900</c:v>
+                  <c:v>930</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4211,7 +4214,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>15 heures 0 minutes</v>
+        <v>15 heures 30 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4228,11 +4231,11 @@
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>900</v>
+        <v>930</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4647,15 +4650,23 @@
       <c r="G21" s="46"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="73" t="str">
+      <c r="A22" s="73">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="36"/>
+        <v>20</v>
+      </c>
+      <c r="B22" s="36">
+        <v>46155</v>
+      </c>
       <c r="C22" s="37"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="28"/>
+      <c r="D22" s="38">
+        <v>30</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="G22" s="45"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -10950,11 +10961,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>900</v>
+        <v>930</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10962,7 +10973,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>15 h 00 min</v>
+        <v>15 h 30 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -11061,22 +11072,22 @@
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>900</v>
+        <v>930</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>15 h 00 min</v>
+        <v>15 h 30 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.17045454545454544</v>
+        <v>0.17613636363636365</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
chore (readme) : update du jdt
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_DamienChabal.xlsx
+++ b/Journal-de-Travail_DamienChabal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\P_AppMobile\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damie\Documents\P_AppMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B5BBE0-5299-409B-931F-F01208E9B5B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26C0C940-B2D2-46D5-96D5-2C3DE7D57112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6600" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="2400" yWindow="795" windowWidth="15060" windowHeight="14295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
   <si>
     <t>Auteur:</t>
   </si>
@@ -179,6 +179,12 @@
   </si>
   <si>
     <t>meilleur affichage</t>
+  </si>
+  <si>
+    <t>ajout utilisation de l'api pour backend</t>
+  </si>
+  <si>
+    <t>Ajout de la gestion des tages et filtrage</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1127,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>930</c:v>
+                  <c:v>1050</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1191,6 +1197,7 @@
     </c:legend>
     <c:plotVisOnly val="0"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1198,7 +1205,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1538,6 +1544,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1545,7 +1552,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2134,6 +2140,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2141,7 +2148,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4214,7 +4220,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>15 heures 30 minutes</v>
+        <v>17 heures 30 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4227,7 +4233,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>660</v>
+        <v>780</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4235,7 +4241,7 @@
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>930</v>
+        <v>1050</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4670,27 +4676,43 @@
       <c r="G22" s="45"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="74" t="str">
+      <c r="A23" s="74">
         <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="40"/>
-      <c r="C23" s="41"/>
+        <v>22</v>
+      </c>
+      <c r="B23" s="40">
+        <v>46167</v>
+      </c>
+      <c r="C23" s="41">
+        <v>1</v>
+      </c>
       <c r="D23" s="42"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="28"/>
+      <c r="E23" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="28" t="s">
+        <v>46</v>
+      </c>
       <c r="G23" s="46"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="73" t="str">
+      <c r="A24" s="73">
         <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
+        <v>22</v>
+      </c>
+      <c r="B24" s="36">
+        <v>46167</v>
+      </c>
+      <c r="C24" s="37">
+        <v>1</v>
+      </c>
       <c r="D24" s="38"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="28"/>
+      <c r="E24" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="28" t="s">
+        <v>47</v>
+      </c>
       <c r="G24" s="45"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -10957,7 +10979,7 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>660</v>
+        <v>780</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
@@ -10965,7 +10987,7 @@
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>930</v>
+        <v>1050</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10973,7 +10995,7 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>15 h 30 min</v>
+        <v>17 h 30 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
@@ -11068,7 +11090,7 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>660</v>
+        <v>780</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
@@ -11076,18 +11098,18 @@
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>930</v>
+        <v>1050</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>15 h 30 min</v>
+        <v>17 h 30 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.17613636363636365</v>
+        <v>0.19886363636363635</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11126,6 +11148,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010080C9F2488912074FB587B9AD9ADAE5BB" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="020ab319e6f8d23aec07c29d6516d4ba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xmlns:ns3="eefa3612-053e-497a-ae76-8a76877f5e22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e15d3f914bf2a775f9387e5284d9197" ns2:_="" ns3:_="">
     <xsd:import namespace="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
@@ -11338,42 +11381,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6394C10-4386-493D-A99B-15992834CB10}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11392,9 +11403,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6394C10-4386-493D-A99B-15992834CB10}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>